<commit_message>
SPM-67 Correct TC09: an Operations Manager has no Venue tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-67_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-67_Test_Cases.xlsx
@@ -1355,7 +1355,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
+    <row r="5" ht="98.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1365,7 +1365,8 @@
         <is>
           <t>1. Log in as grace.lim@connectsphere.com / password123
 2. Click 'All Events' in the sidebar and open 'SPM67 Status Mix'
-3. Click the 'Venue' tab</t>
+3. Note the event reference shown next to the title
+4. Type /events/&lt;reference from step 3&gt;/venue after the site address in the browser address bar (e.g. http://localhost:3000/events/&lt;reference from step 3&gt;/venue) and press Enter</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1383,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="58" customHeight="1">
+    <row r="7" ht="139" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1390,7 +1391,8 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 3: A blue alert reads 'Only the assigned Coordinator can request a venue booking.' The 'Booking requests' card lists all five rows with their badges, but no row has a 'Withdraw request' or 'Release booking' button.</t>
+          <t>Step 2: The event opens on its Overview. The tab bar has 'Overview' only: an Operations Manager has no 'Venue' tab. The 'Venue bookings' card lists the approved SPM67 Studio booking, and there is no 'Withdraw request' or 'Release booking' button anywhere on the page.
+Step 4: The event's 'Find a venue' page opens. A blue alert reads 'Only the assigned Coordinator can request a venue booking.' The 'Booking requests' card lists all five rows with their badges, but no row has a 'Withdraw request' or 'Release booking' button.</t>
         </is>
       </c>
     </row>
@@ -1744,13 +1746,13 @@
       </c>
       <c r="C7" s="11" t="n"/>
     </row>
-    <row r="8" ht="125.5" customHeight="1">
+    <row r="8" ht="179.5" customHeight="1">
       <c r="A8" s="11" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-11 (AC9): who may see the buttons follows the request rule (canRequestVenueBooking): only the assigned Coordinator. Other Coordinators, the Ops Manager and Venue Staff see the booking list with the existing message 'Only the assigned Coordinator can request a venue booking.' and no buttons (TC08-TC10). The Event Organiser has no Venue tab (venue:view), so no case is written for them. The API refuses a withdraw or release from anyone else with 'Only the assigned Coordinator can withdraw or release a venue booking.' - reachable only by calling the API, so unit-tested, not a case.</t>
+          <t>DECIDED 2026-10-11 (AC9): who may see the buttons follows the request rule (canRequestVenueBooking): only the assigned Coordinator. Other Coordinators, the Ops Manager and Venue Staff see the booking list with the existing message 'Only the assigned Coordinator can request a venue booking.' and no buttons (TC08-TC10). The Event Organiser has no Venue tab (venue:view), so no case is written for them. The API refuses a withdraw or release from anyone else with 'Only the assigned Coordinator can withdraw or release a venue booking.' - reachable only by calling the API, so unit-tested, not a case. Corrected 2026-10-13 during the manual pass: an Operations Manager has no Venue tab (EVENT_TABS_BY_ROLE in src/lib/roles.ts), so TC09 now checks the Overview and then opens the Venue page by its address, as TC10 does for Venue Staff. The case was wrong, not the app.</t>
         </is>
       </c>
       <c r="C8" s="11" t="n"/>

</xml_diff>

<commit_message>
SPM-67 Record the manual test pass; changelog, Known Gaps and UI design
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-67_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-67_Test_Cases.xlsx
@@ -1680,13 +1680,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="179.5" customHeight="1">
+    <row r="2" ht="206.5" customHeight="1">
       <c r="A2" s="11" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Written 2026-10-11 before any SPM-67 code (test-first), then checked against the built code the same day (kayalvizhi24): every label, dialog, message and badge quoted in the cases is what the Venue tab now shows. Fixture dates were moved from September to November 2027 while building, because the app writes September as 'Sept' (en-SG), so a quoted 'Sep' would not match the screen. Built: PATCH /api/events/[id]/venue-bookings/[bookingId] (withdraw or release), src/lib/venueBookingChange.ts (the rules and the Venue Staff notification), the Venue tab's buttons and dialog, the 'Released' badge, and migration 20261011120000_add_venue_booking_withdrawal (to apply with `npx prisma migrate deploy`, no reseed; `npm run fixtures:spm67` needs it applied first). No case was added from code: the only behaviour beyond the ACs (two people acting on one booking at once, a closed event) is unit-tested.</t>
+          <t>Written 2026-10-11 before any SPM-67 code (test-first), then checked against the built code the same day (kayalvizhi24): every label, dialog, message and badge quoted in the cases is what the Venue tab now shows. Fixture dates were moved from September to November 2027 while building, because the app writes September as 'Sept' (en-SG), so a quoted 'Sep' would not match the screen. Built: PATCH /api/events/[id]/venue-bookings/[bookingId] (withdraw or release), src/lib/venueBookingChange.ts (the rules and the Venue Staff notification), the Venue tab's buttons and dialog, the 'Released' badge, and migration 20261011120000_add_venue_booking_withdrawal (applied to the shared database with `prisma migrate deploy`, no reseed). No case was added from code: the only behaviour beyond the ACs (two people acting on one booking at once, a closed event) is unit-tested. All 10 cases passed when run by hand on 2026-10-13 (kayalvizhi24), on the build with main merged in (SPM-33, SPM-55, SPM-64, SPM-85).</t>
         </is>
       </c>
       <c r="C2" s="11" t="n"/>

</xml_diff>